<commit_message>
added data to creek and seminole
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Creek/Creek Freedman Minor.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Creek/Creek Freedman Minor.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="17">
   <si>
     <t>ID</t>
   </si>
@@ -59,6 +59,12 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>Creek</t>
+  </si>
+  <si>
+    <t>Freedman (Minor)</t>
   </si>
 </sst>
 </file>
@@ -392,6 +398,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O330"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="12" max="12" width="17.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" t="s">
@@ -444,1973 +453,3947 @@
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
       </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4">
         <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L5" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="L7" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L8" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="L9" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L12" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="L14" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1">
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="L16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1">
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="L17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1">
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="L18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1">
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="L19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1">
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+      <c r="L20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1">
+      <c r="B21" t="s">
+        <v>15</v>
+      </c>
+      <c r="L21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1">
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+      <c r="L22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1">
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="L23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1">
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+      <c r="L24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1">
+      <c r="B25" t="s">
+        <v>15</v>
+      </c>
+      <c r="L25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:1">
+      <c r="B26" t="s">
+        <v>15</v>
+      </c>
+      <c r="L26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:1">
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+      <c r="L27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1">
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="L28" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:1">
+      <c r="B29" t="s">
+        <v>15</v>
+      </c>
+      <c r="L29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:1">
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+      <c r="L30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:1">
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="L31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1">
+      <c r="B32" t="s">
+        <v>15</v>
+      </c>
+      <c r="L32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
       <c r="A33">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1">
+      <c r="B33" t="s">
+        <v>15</v>
+      </c>
+      <c r="L33" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
       <c r="A34">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1">
+      <c r="B34" t="s">
+        <v>15</v>
+      </c>
+      <c r="L34" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
       <c r="A35">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1">
+      <c r="B35" t="s">
+        <v>15</v>
+      </c>
+      <c r="L35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
       <c r="A36">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:1">
+      <c r="B36" t="s">
+        <v>15</v>
+      </c>
+      <c r="L36" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
       <c r="A37">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:1">
+      <c r="B37" t="s">
+        <v>15</v>
+      </c>
+      <c r="L37" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
       <c r="A38">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:1">
+      <c r="B38" t="s">
+        <v>15</v>
+      </c>
+      <c r="L38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
       <c r="A39">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:1">
+      <c r="B39" t="s">
+        <v>15</v>
+      </c>
+      <c r="L39" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
       <c r="A40">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:1">
+      <c r="B40" t="s">
+        <v>15</v>
+      </c>
+      <c r="L40" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
       <c r="A41">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1">
+      <c r="B41" t="s">
+        <v>15</v>
+      </c>
+      <c r="L41" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
       <c r="A42">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-    </row>
-    <row r="43" spans="1:1">
+      <c r="B42" t="s">
+        <v>15</v>
+      </c>
+      <c r="L42" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
       <c r="A43">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-    </row>
-    <row r="44" spans="1:1">
+      <c r="B43" t="s">
+        <v>15</v>
+      </c>
+      <c r="L43" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12">
       <c r="A44">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:1">
+      <c r="B44" t="s">
+        <v>15</v>
+      </c>
+      <c r="L44" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-    </row>
-    <row r="46" spans="1:1">
+      <c r="B45" t="s">
+        <v>15</v>
+      </c>
+      <c r="L45" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12">
       <c r="A46">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-    </row>
-    <row r="47" spans="1:1">
+      <c r="B46" t="s">
+        <v>15</v>
+      </c>
+      <c r="L46" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12">
       <c r="A47">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:1">
+      <c r="B47" t="s">
+        <v>15</v>
+      </c>
+      <c r="L47" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12">
       <c r="A48">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:1">
+      <c r="B48" t="s">
+        <v>15</v>
+      </c>
+      <c r="L48" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
       <c r="A49">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:1">
+      <c r="B49" t="s">
+        <v>15</v>
+      </c>
+      <c r="L49" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
       <c r="A50">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:1">
+      <c r="B50" t="s">
+        <v>15</v>
+      </c>
+      <c r="L50" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
       <c r="A51">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-    </row>
-    <row r="52" spans="1:1">
+      <c r="B51" t="s">
+        <v>15</v>
+      </c>
+      <c r="L51" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
       <c r="A52">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-    </row>
-    <row r="53" spans="1:1">
+      <c r="B52" t="s">
+        <v>15</v>
+      </c>
+      <c r="L52" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12">
       <c r="A53">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-    </row>
-    <row r="54" spans="1:1">
+      <c r="B53" t="s">
+        <v>15</v>
+      </c>
+      <c r="L53" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12">
       <c r="A54">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-    </row>
-    <row r="55" spans="1:1">
+      <c r="B54" t="s">
+        <v>15</v>
+      </c>
+      <c r="L54" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12">
       <c r="A55">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-    </row>
-    <row r="56" spans="1:1">
+      <c r="B55" t="s">
+        <v>15</v>
+      </c>
+      <c r="L55" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12">
       <c r="A56">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-    </row>
-    <row r="57" spans="1:1">
+      <c r="B56" t="s">
+        <v>15</v>
+      </c>
+      <c r="L56" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12">
       <c r="A57">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-    </row>
-    <row r="58" spans="1:1">
+      <c r="B57" t="s">
+        <v>15</v>
+      </c>
+      <c r="L57" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12">
       <c r="A58">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-    </row>
-    <row r="59" spans="1:1">
+      <c r="B58" t="s">
+        <v>15</v>
+      </c>
+      <c r="L58" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12">
       <c r="A59">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-    </row>
-    <row r="60" spans="1:1">
+      <c r="B59" t="s">
+        <v>15</v>
+      </c>
+      <c r="L59" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12">
       <c r="A60">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-    </row>
-    <row r="61" spans="1:1">
+      <c r="B60" t="s">
+        <v>15</v>
+      </c>
+      <c r="L60" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12">
       <c r="A61">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-    </row>
-    <row r="62" spans="1:1">
+      <c r="B61" t="s">
+        <v>15</v>
+      </c>
+      <c r="L61" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12">
       <c r="A62">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-    </row>
-    <row r="63" spans="1:1">
+      <c r="B62" t="s">
+        <v>15</v>
+      </c>
+      <c r="L62" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12">
       <c r="A63">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-    </row>
-    <row r="64" spans="1:1">
+      <c r="B63" t="s">
+        <v>15</v>
+      </c>
+      <c r="L63" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12">
       <c r="A64">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-    </row>
-    <row r="65" spans="1:1">
+      <c r="B64" t="s">
+        <v>15</v>
+      </c>
+      <c r="L64" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12">
       <c r="A65">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-    </row>
-    <row r="66" spans="1:1">
+      <c r="B65" t="s">
+        <v>15</v>
+      </c>
+      <c r="L65" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12">
       <c r="A66">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
-    </row>
-    <row r="67" spans="1:1">
+      <c r="B66" t="s">
+        <v>15</v>
+      </c>
+      <c r="L66" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12">
       <c r="A67">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-    </row>
-    <row r="68" spans="1:1">
+      <c r="B67" t="s">
+        <v>15</v>
+      </c>
+      <c r="L67" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12">
       <c r="A68">
         <f t="shared" ref="A68:A131" si="1">A67+1</f>
         <v>67</v>
       </c>
-    </row>
-    <row r="69" spans="1:1">
+      <c r="B68" t="s">
+        <v>15</v>
+      </c>
+      <c r="L68" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12">
       <c r="A69">
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-    </row>
-    <row r="70" spans="1:1">
+      <c r="B69" t="s">
+        <v>15</v>
+      </c>
+      <c r="L69" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12">
       <c r="A70">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-    </row>
-    <row r="71" spans="1:1">
+      <c r="B70" t="s">
+        <v>15</v>
+      </c>
+      <c r="L70" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12">
       <c r="A71">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-    </row>
-    <row r="72" spans="1:1">
+      <c r="B71" t="s">
+        <v>15</v>
+      </c>
+      <c r="L71" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12">
       <c r="A72">
         <f t="shared" si="1"/>
         <v>71</v>
       </c>
-    </row>
-    <row r="73" spans="1:1">
+      <c r="B72" t="s">
+        <v>15</v>
+      </c>
+      <c r="L72" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12">
       <c r="A73">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-    </row>
-    <row r="74" spans="1:1">
+      <c r="B73" t="s">
+        <v>15</v>
+      </c>
+      <c r="L73" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12">
       <c r="A74">
         <f t="shared" si="1"/>
         <v>73</v>
       </c>
-    </row>
-    <row r="75" spans="1:1">
+      <c r="B74" t="s">
+        <v>15</v>
+      </c>
+      <c r="L74" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12">
       <c r="A75">
         <f t="shared" si="1"/>
         <v>74</v>
       </c>
-    </row>
-    <row r="76" spans="1:1">
+      <c r="B75" t="s">
+        <v>15</v>
+      </c>
+      <c r="L75" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12">
       <c r="A76">
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
-    </row>
-    <row r="77" spans="1:1">
+      <c r="B76" t="s">
+        <v>15</v>
+      </c>
+      <c r="L76" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12">
       <c r="A77">
         <f t="shared" si="1"/>
         <v>76</v>
       </c>
-    </row>
-    <row r="78" spans="1:1">
+      <c r="B77" t="s">
+        <v>15</v>
+      </c>
+      <c r="L77" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12">
       <c r="A78">
         <f t="shared" si="1"/>
         <v>77</v>
       </c>
-    </row>
-    <row r="79" spans="1:1">
+      <c r="B78" t="s">
+        <v>15</v>
+      </c>
+      <c r="L78" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12">
       <c r="A79">
         <f t="shared" si="1"/>
         <v>78</v>
       </c>
-    </row>
-    <row r="80" spans="1:1">
+      <c r="B79" t="s">
+        <v>15</v>
+      </c>
+      <c r="L79" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12">
       <c r="A80">
         <f t="shared" si="1"/>
         <v>79</v>
       </c>
-    </row>
-    <row r="81" spans="1:1">
+      <c r="B80" t="s">
+        <v>15</v>
+      </c>
+      <c r="L80" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12">
       <c r="A81">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-    </row>
-    <row r="82" spans="1:1">
+      <c r="B81" t="s">
+        <v>15</v>
+      </c>
+      <c r="L81" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12">
       <c r="A82">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
-    </row>
-    <row r="83" spans="1:1">
+      <c r="B82" t="s">
+        <v>15</v>
+      </c>
+      <c r="L82" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12">
       <c r="A83">
         <f t="shared" si="1"/>
         <v>82</v>
       </c>
-    </row>
-    <row r="84" spans="1:1">
+      <c r="B83" t="s">
+        <v>15</v>
+      </c>
+      <c r="L83" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12">
       <c r="A84">
         <f t="shared" si="1"/>
         <v>83</v>
       </c>
-    </row>
-    <row r="85" spans="1:1">
+      <c r="B84" t="s">
+        <v>15</v>
+      </c>
+      <c r="L84" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12">
       <c r="A85">
         <f t="shared" si="1"/>
         <v>84</v>
       </c>
-    </row>
-    <row r="86" spans="1:1">
+      <c r="B85" t="s">
+        <v>15</v>
+      </c>
+      <c r="L85" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12">
       <c r="A86">
         <f t="shared" si="1"/>
         <v>85</v>
       </c>
-    </row>
-    <row r="87" spans="1:1">
+      <c r="B86" t="s">
+        <v>15</v>
+      </c>
+      <c r="L86" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12">
       <c r="A87">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
-    </row>
-    <row r="88" spans="1:1">
+      <c r="B87" t="s">
+        <v>15</v>
+      </c>
+      <c r="L87" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12">
       <c r="A88">
         <f t="shared" si="1"/>
         <v>87</v>
       </c>
-    </row>
-    <row r="89" spans="1:1">
+      <c r="B88" t="s">
+        <v>15</v>
+      </c>
+      <c r="L88" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12">
       <c r="A89">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-    </row>
-    <row r="90" spans="1:1">
+      <c r="B89" t="s">
+        <v>15</v>
+      </c>
+      <c r="L89" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12">
       <c r="A90">
         <f t="shared" si="1"/>
         <v>89</v>
       </c>
-    </row>
-    <row r="91" spans="1:1">
+      <c r="B90" t="s">
+        <v>15</v>
+      </c>
+      <c r="L90" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12">
       <c r="A91">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-    </row>
-    <row r="92" spans="1:1">
+      <c r="B91" t="s">
+        <v>15</v>
+      </c>
+      <c r="L91" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12">
       <c r="A92">
         <f t="shared" si="1"/>
         <v>91</v>
       </c>
-    </row>
-    <row r="93" spans="1:1">
+      <c r="B92" t="s">
+        <v>15</v>
+      </c>
+      <c r="L92" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12">
       <c r="A93">
         <f t="shared" si="1"/>
         <v>92</v>
       </c>
-    </row>
-    <row r="94" spans="1:1">
+      <c r="B93" t="s">
+        <v>15</v>
+      </c>
+      <c r="L93" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12">
       <c r="A94">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-    </row>
-    <row r="95" spans="1:1">
+      <c r="B94" t="s">
+        <v>15</v>
+      </c>
+      <c r="L94" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12">
       <c r="A95">
         <f t="shared" si="1"/>
         <v>94</v>
       </c>
-    </row>
-    <row r="96" spans="1:1">
+      <c r="B95" t="s">
+        <v>15</v>
+      </c>
+      <c r="L95" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12">
       <c r="A96">
         <f t="shared" si="1"/>
         <v>95</v>
       </c>
-    </row>
-    <row r="97" spans="1:1">
+      <c r="B96" t="s">
+        <v>15</v>
+      </c>
+      <c r="L96" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12">
       <c r="A97">
         <f t="shared" si="1"/>
         <v>96</v>
       </c>
-    </row>
-    <row r="98" spans="1:1">
+      <c r="B97" t="s">
+        <v>15</v>
+      </c>
+      <c r="L97" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12">
       <c r="A98">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-    </row>
-    <row r="99" spans="1:1">
+      <c r="B98" t="s">
+        <v>15</v>
+      </c>
+      <c r="L98" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12">
       <c r="A99">
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
-    </row>
-    <row r="100" spans="1:1">
+      <c r="B99" t="s">
+        <v>15</v>
+      </c>
+      <c r="L99" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12">
       <c r="A100">
         <f t="shared" si="1"/>
         <v>99</v>
       </c>
-    </row>
-    <row r="101" spans="1:1">
+      <c r="B100" t="s">
+        <v>15</v>
+      </c>
+      <c r="L100" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12">
       <c r="A101">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-    </row>
-    <row r="102" spans="1:1">
+      <c r="B101" t="s">
+        <v>15</v>
+      </c>
+      <c r="L101" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12">
       <c r="A102">
         <f t="shared" si="1"/>
         <v>101</v>
       </c>
-    </row>
-    <row r="103" spans="1:1">
+      <c r="B102" t="s">
+        <v>15</v>
+      </c>
+      <c r="L102" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12">
       <c r="A103">
         <f t="shared" si="1"/>
         <v>102</v>
       </c>
-    </row>
-    <row r="104" spans="1:1">
+      <c r="B103" t="s">
+        <v>15</v>
+      </c>
+      <c r="L103" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12">
       <c r="A104">
         <f t="shared" si="1"/>
         <v>103</v>
       </c>
-    </row>
-    <row r="105" spans="1:1">
+      <c r="B104" t="s">
+        <v>15</v>
+      </c>
+      <c r="L104" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12">
       <c r="A105">
         <f t="shared" si="1"/>
         <v>104</v>
       </c>
-    </row>
-    <row r="106" spans="1:1">
+      <c r="B105" t="s">
+        <v>15</v>
+      </c>
+      <c r="L105" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12">
       <c r="A106">
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
-    </row>
-    <row r="107" spans="1:1">
+      <c r="B106" t="s">
+        <v>15</v>
+      </c>
+      <c r="L106" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12">
       <c r="A107">
         <f t="shared" si="1"/>
         <v>106</v>
       </c>
-    </row>
-    <row r="108" spans="1:1">
+      <c r="B107" t="s">
+        <v>15</v>
+      </c>
+      <c r="L107" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12">
       <c r="A108">
         <f t="shared" si="1"/>
         <v>107</v>
       </c>
-    </row>
-    <row r="109" spans="1:1">
+      <c r="B108" t="s">
+        <v>15</v>
+      </c>
+      <c r="L108" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12">
       <c r="A109">
         <f t="shared" si="1"/>
         <v>108</v>
       </c>
-    </row>
-    <row r="110" spans="1:1">
+      <c r="B109" t="s">
+        <v>15</v>
+      </c>
+      <c r="L109" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12">
       <c r="A110">
         <f t="shared" si="1"/>
         <v>109</v>
       </c>
-    </row>
-    <row r="111" spans="1:1">
+      <c r="B110" t="s">
+        <v>15</v>
+      </c>
+      <c r="L110" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12">
       <c r="A111">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-    </row>
-    <row r="112" spans="1:1">
+      <c r="B111" t="s">
+        <v>15</v>
+      </c>
+      <c r="L111" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12">
       <c r="A112">
         <f t="shared" si="1"/>
         <v>111</v>
       </c>
-    </row>
-    <row r="113" spans="1:1">
+      <c r="B112" t="s">
+        <v>15</v>
+      </c>
+      <c r="L112" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12">
       <c r="A113">
         <f t="shared" si="1"/>
         <v>112</v>
       </c>
-    </row>
-    <row r="114" spans="1:1">
+      <c r="B113" t="s">
+        <v>15</v>
+      </c>
+      <c r="L113" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12">
       <c r="A114">
         <f t="shared" si="1"/>
         <v>113</v>
       </c>
-    </row>
-    <row r="115" spans="1:1">
+      <c r="B114" t="s">
+        <v>15</v>
+      </c>
+      <c r="L114" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12">
       <c r="A115">
         <f t="shared" si="1"/>
         <v>114</v>
       </c>
-    </row>
-    <row r="116" spans="1:1">
+      <c r="B115" t="s">
+        <v>15</v>
+      </c>
+      <c r="L115" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12">
       <c r="A116">
         <f t="shared" si="1"/>
         <v>115</v>
       </c>
-    </row>
-    <row r="117" spans="1:1">
+      <c r="B116" t="s">
+        <v>15</v>
+      </c>
+      <c r="L116" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12">
       <c r="A117">
         <f t="shared" si="1"/>
         <v>116</v>
       </c>
-    </row>
-    <row r="118" spans="1:1">
+      <c r="B117" t="s">
+        <v>15</v>
+      </c>
+      <c r="L117" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12">
       <c r="A118">
         <f t="shared" si="1"/>
         <v>117</v>
       </c>
-    </row>
-    <row r="119" spans="1:1">
+      <c r="B118" t="s">
+        <v>15</v>
+      </c>
+      <c r="L118" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12">
       <c r="A119">
         <f t="shared" si="1"/>
         <v>118</v>
       </c>
-    </row>
-    <row r="120" spans="1:1">
+      <c r="B119" t="s">
+        <v>15</v>
+      </c>
+      <c r="L119" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12">
       <c r="A120">
         <f t="shared" si="1"/>
         <v>119</v>
       </c>
-    </row>
-    <row r="121" spans="1:1">
+      <c r="B120" t="s">
+        <v>15</v>
+      </c>
+      <c r="L120" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12">
       <c r="A121">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-    </row>
-    <row r="122" spans="1:1">
+      <c r="B121" t="s">
+        <v>15</v>
+      </c>
+      <c r="L121" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12">
       <c r="A122">
         <f t="shared" si="1"/>
         <v>121</v>
       </c>
-    </row>
-    <row r="123" spans="1:1">
+      <c r="B122" t="s">
+        <v>15</v>
+      </c>
+      <c r="L122" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12">
       <c r="A123">
         <f t="shared" si="1"/>
         <v>122</v>
       </c>
-    </row>
-    <row r="124" spans="1:1">
+      <c r="B123" t="s">
+        <v>15</v>
+      </c>
+      <c r="L123" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12">
       <c r="A124">
         <f t="shared" si="1"/>
         <v>123</v>
       </c>
-    </row>
-    <row r="125" spans="1:1">
+      <c r="B124" t="s">
+        <v>15</v>
+      </c>
+      <c r="L124" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12">
       <c r="A125">
         <f t="shared" si="1"/>
         <v>124</v>
       </c>
-    </row>
-    <row r="126" spans="1:1">
+      <c r="B125" t="s">
+        <v>15</v>
+      </c>
+      <c r="L125" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12">
       <c r="A126">
         <f t="shared" si="1"/>
         <v>125</v>
       </c>
-    </row>
-    <row r="127" spans="1:1">
+      <c r="B126" t="s">
+        <v>15</v>
+      </c>
+      <c r="L126" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12">
       <c r="A127">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-    </row>
-    <row r="128" spans="1:1">
+      <c r="B127" t="s">
+        <v>15</v>
+      </c>
+      <c r="L127" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12">
       <c r="A128">
         <f t="shared" si="1"/>
         <v>127</v>
       </c>
-    </row>
-    <row r="129" spans="1:1">
+      <c r="B128" t="s">
+        <v>15</v>
+      </c>
+      <c r="L128" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12">
       <c r="A129">
         <f t="shared" si="1"/>
         <v>128</v>
       </c>
-    </row>
-    <row r="130" spans="1:1">
+      <c r="B129" t="s">
+        <v>15</v>
+      </c>
+      <c r="L129" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12">
       <c r="A130">
         <f t="shared" si="1"/>
         <v>129</v>
       </c>
-    </row>
-    <row r="131" spans="1:1">
+      <c r="B130" t="s">
+        <v>15</v>
+      </c>
+      <c r="L130" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12">
       <c r="A131">
         <f t="shared" si="1"/>
         <v>130</v>
       </c>
-    </row>
-    <row r="132" spans="1:1">
+      <c r="B131" t="s">
+        <v>15</v>
+      </c>
+      <c r="L131" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12">
       <c r="A132">
         <f t="shared" ref="A132:A195" si="2">A131+1</f>
         <v>131</v>
       </c>
-    </row>
-    <row r="133" spans="1:1">
+      <c r="B132" t="s">
+        <v>15</v>
+      </c>
+      <c r="L132" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12">
       <c r="A133">
         <f t="shared" si="2"/>
         <v>132</v>
       </c>
-    </row>
-    <row r="134" spans="1:1">
+      <c r="B133" t="s">
+        <v>15</v>
+      </c>
+      <c r="L133" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12">
       <c r="A134">
         <f t="shared" si="2"/>
         <v>133</v>
       </c>
-    </row>
-    <row r="135" spans="1:1">
+      <c r="B134" t="s">
+        <v>15</v>
+      </c>
+      <c r="L134" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12">
       <c r="A135">
         <f t="shared" si="2"/>
         <v>134</v>
       </c>
-    </row>
-    <row r="136" spans="1:1">
+      <c r="B135" t="s">
+        <v>15</v>
+      </c>
+      <c r="L135" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12">
       <c r="A136">
         <f t="shared" si="2"/>
         <v>135</v>
       </c>
-    </row>
-    <row r="137" spans="1:1">
+      <c r="B136" t="s">
+        <v>15</v>
+      </c>
+      <c r="L136" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12">
       <c r="A137">
         <f t="shared" si="2"/>
         <v>136</v>
       </c>
-    </row>
-    <row r="138" spans="1:1">
+      <c r="B137" t="s">
+        <v>15</v>
+      </c>
+      <c r="L137" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12">
       <c r="A138">
         <f t="shared" si="2"/>
         <v>137</v>
       </c>
-    </row>
-    <row r="139" spans="1:1">
+      <c r="B138" t="s">
+        <v>15</v>
+      </c>
+      <c r="L138" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12">
       <c r="A139">
         <f t="shared" si="2"/>
         <v>138</v>
       </c>
-    </row>
-    <row r="140" spans="1:1">
+      <c r="B139" t="s">
+        <v>15</v>
+      </c>
+      <c r="L139" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12">
       <c r="A140">
         <f t="shared" si="2"/>
         <v>139</v>
       </c>
-    </row>
-    <row r="141" spans="1:1">
+      <c r="B140" t="s">
+        <v>15</v>
+      </c>
+      <c r="L140" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12">
       <c r="A141">
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
-    </row>
-    <row r="142" spans="1:1">
+      <c r="B141" t="s">
+        <v>15</v>
+      </c>
+      <c r="L141" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12">
       <c r="A142">
         <f t="shared" si="2"/>
         <v>141</v>
       </c>
-    </row>
-    <row r="143" spans="1:1">
+      <c r="B142" t="s">
+        <v>15</v>
+      </c>
+      <c r="L142" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12">
       <c r="A143">
         <f t="shared" si="2"/>
         <v>142</v>
       </c>
-    </row>
-    <row r="144" spans="1:1">
+      <c r="B143" t="s">
+        <v>15</v>
+      </c>
+      <c r="L143" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12">
       <c r="A144">
         <f t="shared" si="2"/>
         <v>143</v>
       </c>
-    </row>
-    <row r="145" spans="1:1">
+      <c r="B144" t="s">
+        <v>15</v>
+      </c>
+      <c r="L144" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="145" spans="1:12">
       <c r="A145">
         <f t="shared" si="2"/>
         <v>144</v>
       </c>
-    </row>
-    <row r="146" spans="1:1">
+      <c r="B145" t="s">
+        <v>15</v>
+      </c>
+      <c r="L145" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12">
       <c r="A146">
         <f t="shared" si="2"/>
         <v>145</v>
       </c>
-    </row>
-    <row r="147" spans="1:1">
+      <c r="B146" t="s">
+        <v>15</v>
+      </c>
+      <c r="L146" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="147" spans="1:12">
       <c r="A147">
         <f t="shared" si="2"/>
         <v>146</v>
       </c>
-    </row>
-    <row r="148" spans="1:1">
+      <c r="B147" t="s">
+        <v>15</v>
+      </c>
+      <c r="L147" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12">
       <c r="A148">
         <f t="shared" si="2"/>
         <v>147</v>
       </c>
-    </row>
-    <row r="149" spans="1:1">
+      <c r="B148" t="s">
+        <v>15</v>
+      </c>
+      <c r="L148" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="149" spans="1:12">
       <c r="A149">
         <f t="shared" si="2"/>
         <v>148</v>
       </c>
-    </row>
-    <row r="150" spans="1:1">
+      <c r="B149" t="s">
+        <v>15</v>
+      </c>
+      <c r="L149" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12">
       <c r="A150">
         <f t="shared" si="2"/>
         <v>149</v>
       </c>
-    </row>
-    <row r="151" spans="1:1">
+      <c r="B150" t="s">
+        <v>15</v>
+      </c>
+      <c r="L150" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12">
       <c r="A151">
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
-    </row>
-    <row r="152" spans="1:1">
+      <c r="B151" t="s">
+        <v>15</v>
+      </c>
+      <c r="L151" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="152" spans="1:12">
       <c r="A152">
         <f t="shared" si="2"/>
         <v>151</v>
       </c>
-    </row>
-    <row r="153" spans="1:1">
+      <c r="B152" t="s">
+        <v>15</v>
+      </c>
+      <c r="L152" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12">
       <c r="A153">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
-    </row>
-    <row r="154" spans="1:1">
+      <c r="B153" t="s">
+        <v>15</v>
+      </c>
+      <c r="L153" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12">
       <c r="A154">
         <f t="shared" si="2"/>
         <v>153</v>
       </c>
-    </row>
-    <row r="155" spans="1:1">
+      <c r="B154" t="s">
+        <v>15</v>
+      </c>
+      <c r="L154" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12">
       <c r="A155">
         <f t="shared" si="2"/>
         <v>154</v>
       </c>
-    </row>
-    <row r="156" spans="1:1">
+      <c r="B155" t="s">
+        <v>15</v>
+      </c>
+      <c r="L155" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12">
       <c r="A156">
         <f t="shared" si="2"/>
         <v>155</v>
       </c>
-    </row>
-    <row r="157" spans="1:1">
+      <c r="B156" t="s">
+        <v>15</v>
+      </c>
+      <c r="L156" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="157" spans="1:12">
       <c r="A157">
         <f t="shared" si="2"/>
         <v>156</v>
       </c>
-    </row>
-    <row r="158" spans="1:1">
+      <c r="B157" t="s">
+        <v>15</v>
+      </c>
+      <c r="L157" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12">
       <c r="A158">
         <f t="shared" si="2"/>
         <v>157</v>
       </c>
-    </row>
-    <row r="159" spans="1:1">
+      <c r="B158" t="s">
+        <v>15</v>
+      </c>
+      <c r="L158" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="159" spans="1:12">
       <c r="A159">
         <f t="shared" si="2"/>
         <v>158</v>
       </c>
-    </row>
-    <row r="160" spans="1:1">
+      <c r="B159" t="s">
+        <v>15</v>
+      </c>
+      <c r="L159" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12">
       <c r="A160">
         <f t="shared" si="2"/>
         <v>159</v>
       </c>
-    </row>
-    <row r="161" spans="1:1">
+      <c r="B160" t="s">
+        <v>15</v>
+      </c>
+      <c r="L160" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12">
       <c r="A161">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-    </row>
-    <row r="162" spans="1:1">
+      <c r="B161" t="s">
+        <v>15</v>
+      </c>
+      <c r="L161" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12">
       <c r="A162">
         <f t="shared" si="2"/>
         <v>161</v>
       </c>
-    </row>
-    <row r="163" spans="1:1">
+      <c r="B162" t="s">
+        <v>15</v>
+      </c>
+      <c r="L162" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12">
       <c r="A163">
         <f t="shared" si="2"/>
         <v>162</v>
       </c>
-    </row>
-    <row r="164" spans="1:1">
+      <c r="B163" t="s">
+        <v>15</v>
+      </c>
+      <c r="L163" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12">
       <c r="A164">
         <f t="shared" si="2"/>
         <v>163</v>
       </c>
-    </row>
-    <row r="165" spans="1:1">
+      <c r="B164" t="s">
+        <v>15</v>
+      </c>
+      <c r="L164" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="165" spans="1:12">
       <c r="A165">
         <f t="shared" si="2"/>
         <v>164</v>
       </c>
-    </row>
-    <row r="166" spans="1:1">
+      <c r="B165" t="s">
+        <v>15</v>
+      </c>
+      <c r="L165" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12">
       <c r="A166">
         <f t="shared" si="2"/>
         <v>165</v>
       </c>
-    </row>
-    <row r="167" spans="1:1">
+      <c r="B166" t="s">
+        <v>15</v>
+      </c>
+      <c r="L166" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="167" spans="1:12">
       <c r="A167">
         <f t="shared" si="2"/>
         <v>166</v>
       </c>
-    </row>
-    <row r="168" spans="1:1">
+      <c r="B167" t="s">
+        <v>15</v>
+      </c>
+      <c r="L167" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12">
       <c r="A168">
         <f t="shared" si="2"/>
         <v>167</v>
       </c>
-    </row>
-    <row r="169" spans="1:1">
+      <c r="B168" t="s">
+        <v>15</v>
+      </c>
+      <c r="L168" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="169" spans="1:12">
       <c r="A169">
         <f t="shared" si="2"/>
         <v>168</v>
       </c>
-    </row>
-    <row r="170" spans="1:1">
+      <c r="B169" t="s">
+        <v>15</v>
+      </c>
+      <c r="L169" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="170" spans="1:12">
       <c r="A170">
         <f t="shared" si="2"/>
         <v>169</v>
       </c>
-    </row>
-    <row r="171" spans="1:1">
+      <c r="B170" t="s">
+        <v>15</v>
+      </c>
+      <c r="L170" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12">
       <c r="A171">
         <f t="shared" si="2"/>
         <v>170</v>
       </c>
-    </row>
-    <row r="172" spans="1:1">
+      <c r="B171" t="s">
+        <v>15</v>
+      </c>
+      <c r="L171" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="172" spans="1:12">
       <c r="A172">
         <f t="shared" si="2"/>
         <v>171</v>
       </c>
-    </row>
-    <row r="173" spans="1:1">
+      <c r="B172" t="s">
+        <v>15</v>
+      </c>
+      <c r="L172" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12">
       <c r="A173">
         <f t="shared" si="2"/>
         <v>172</v>
       </c>
-    </row>
-    <row r="174" spans="1:1">
+      <c r="B173" t="s">
+        <v>15</v>
+      </c>
+      <c r="L173" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="174" spans="1:12">
       <c r="A174">
         <f t="shared" si="2"/>
         <v>173</v>
       </c>
-    </row>
-    <row r="175" spans="1:1">
+      <c r="B174" t="s">
+        <v>15</v>
+      </c>
+      <c r="L174" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12">
       <c r="A175">
         <f t="shared" si="2"/>
         <v>174</v>
       </c>
-    </row>
-    <row r="176" spans="1:1">
+      <c r="B175" t="s">
+        <v>15</v>
+      </c>
+      <c r="L175" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12">
       <c r="A176">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
-    </row>
-    <row r="177" spans="1:1">
+      <c r="B176" t="s">
+        <v>15</v>
+      </c>
+      <c r="L176" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="177" spans="1:12">
       <c r="A177">
         <f t="shared" si="2"/>
         <v>176</v>
       </c>
-    </row>
-    <row r="178" spans="1:1">
+      <c r="B177" t="s">
+        <v>15</v>
+      </c>
+      <c r="L177" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="178" spans="1:12">
       <c r="A178">
         <f t="shared" si="2"/>
         <v>177</v>
       </c>
-    </row>
-    <row r="179" spans="1:1">
+      <c r="B178" t="s">
+        <v>15</v>
+      </c>
+      <c r="L178" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12">
       <c r="A179">
         <f t="shared" si="2"/>
         <v>178</v>
       </c>
-    </row>
-    <row r="180" spans="1:1">
+      <c r="B179" t="s">
+        <v>15</v>
+      </c>
+      <c r="L179" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="180" spans="1:12">
       <c r="A180">
         <f t="shared" si="2"/>
         <v>179</v>
       </c>
-    </row>
-    <row r="181" spans="1:1">
+      <c r="B180" t="s">
+        <v>15</v>
+      </c>
+      <c r="L180" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="181" spans="1:12">
       <c r="A181">
         <f t="shared" si="2"/>
         <v>180</v>
       </c>
-    </row>
-    <row r="182" spans="1:1">
+      <c r="B181" t="s">
+        <v>15</v>
+      </c>
+      <c r="L181" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12">
       <c r="A182">
         <f t="shared" si="2"/>
         <v>181</v>
       </c>
-    </row>
-    <row r="183" spans="1:1">
+      <c r="B182" t="s">
+        <v>15</v>
+      </c>
+      <c r="L182" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12">
       <c r="A183">
         <f t="shared" si="2"/>
         <v>182</v>
       </c>
-    </row>
-    <row r="184" spans="1:1">
+      <c r="B183" t="s">
+        <v>15</v>
+      </c>
+      <c r="L183" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12">
       <c r="A184">
         <f t="shared" si="2"/>
         <v>183</v>
       </c>
-    </row>
-    <row r="185" spans="1:1">
+      <c r="B184" t="s">
+        <v>15</v>
+      </c>
+      <c r="L184" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12">
       <c r="A185">
         <f t="shared" si="2"/>
         <v>184</v>
       </c>
-    </row>
-    <row r="186" spans="1:1">
+      <c r="B185" t="s">
+        <v>15</v>
+      </c>
+      <c r="L185" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="186" spans="1:12">
       <c r="A186">
         <f t="shared" si="2"/>
         <v>185</v>
       </c>
-    </row>
-    <row r="187" spans="1:1">
+      <c r="B186" t="s">
+        <v>15</v>
+      </c>
+      <c r="L186" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="187" spans="1:12">
       <c r="A187">
         <f t="shared" si="2"/>
         <v>186</v>
       </c>
-    </row>
-    <row r="188" spans="1:1">
+      <c r="B187" t="s">
+        <v>15</v>
+      </c>
+      <c r="L187" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="188" spans="1:12">
       <c r="A188">
         <f t="shared" si="2"/>
         <v>187</v>
       </c>
-    </row>
-    <row r="189" spans="1:1">
+      <c r="B188" t="s">
+        <v>15</v>
+      </c>
+      <c r="L188" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="189" spans="1:12">
       <c r="A189">
         <f t="shared" si="2"/>
         <v>188</v>
       </c>
-    </row>
-    <row r="190" spans="1:1">
+      <c r="B189" t="s">
+        <v>15</v>
+      </c>
+      <c r="L189" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="190" spans="1:12">
       <c r="A190">
         <f t="shared" si="2"/>
         <v>189</v>
       </c>
-    </row>
-    <row r="191" spans="1:1">
+      <c r="B190" t="s">
+        <v>15</v>
+      </c>
+      <c r="L190" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="191" spans="1:12">
       <c r="A191">
         <f t="shared" si="2"/>
         <v>190</v>
       </c>
-    </row>
-    <row r="192" spans="1:1">
+      <c r="B191" t="s">
+        <v>15</v>
+      </c>
+      <c r="L191" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="192" spans="1:12">
       <c r="A192">
         <f t="shared" si="2"/>
         <v>191</v>
       </c>
-    </row>
-    <row r="193" spans="1:1">
+      <c r="B192" t="s">
+        <v>15</v>
+      </c>
+      <c r="L192" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="193" spans="1:12">
       <c r="A193">
         <f t="shared" si="2"/>
         <v>192</v>
       </c>
-    </row>
-    <row r="194" spans="1:1">
+      <c r="B193" t="s">
+        <v>15</v>
+      </c>
+      <c r="L193" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12">
       <c r="A194">
         <f t="shared" si="2"/>
         <v>193</v>
       </c>
-    </row>
-    <row r="195" spans="1:1">
+      <c r="B194" t="s">
+        <v>15</v>
+      </c>
+      <c r="L194" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12">
       <c r="A195">
         <f t="shared" si="2"/>
         <v>194</v>
       </c>
-    </row>
-    <row r="196" spans="1:1">
+      <c r="B195" t="s">
+        <v>15</v>
+      </c>
+      <c r="L195" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12">
       <c r="A196">
         <f t="shared" ref="A196:A259" si="3">A195+1</f>
         <v>195</v>
       </c>
-    </row>
-    <row r="197" spans="1:1">
+      <c r="B196" t="s">
+        <v>15</v>
+      </c>
+      <c r="L196" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="197" spans="1:12">
       <c r="A197">
         <f t="shared" si="3"/>
         <v>196</v>
       </c>
-    </row>
-    <row r="198" spans="1:1">
+      <c r="B197" t="s">
+        <v>15</v>
+      </c>
+      <c r="L197" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12">
       <c r="A198">
         <f t="shared" si="3"/>
         <v>197</v>
       </c>
-    </row>
-    <row r="199" spans="1:1">
+      <c r="B198" t="s">
+        <v>15</v>
+      </c>
+      <c r="L198" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="199" spans="1:12">
       <c r="A199">
         <f t="shared" si="3"/>
         <v>198</v>
       </c>
-    </row>
-    <row r="200" spans="1:1">
+      <c r="B199" t="s">
+        <v>15</v>
+      </c>
+      <c r="L199" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12">
       <c r="A200">
         <f t="shared" si="3"/>
         <v>199</v>
       </c>
-    </row>
-    <row r="201" spans="1:1">
+      <c r="B200" t="s">
+        <v>15</v>
+      </c>
+      <c r="L200" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="201" spans="1:12">
       <c r="A201">
         <f t="shared" si="3"/>
         <v>200</v>
       </c>
-    </row>
-    <row r="202" spans="1:1">
+      <c r="B201" t="s">
+        <v>15</v>
+      </c>
+      <c r="L201" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12">
       <c r="A202">
         <f t="shared" si="3"/>
         <v>201</v>
       </c>
-    </row>
-    <row r="203" spans="1:1">
+      <c r="B202" t="s">
+        <v>15</v>
+      </c>
+      <c r="L202" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="203" spans="1:12">
       <c r="A203">
         <f t="shared" si="3"/>
         <v>202</v>
       </c>
-    </row>
-    <row r="204" spans="1:1">
+      <c r="B203" t="s">
+        <v>15</v>
+      </c>
+      <c r="L203" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="204" spans="1:12">
       <c r="A204">
         <f t="shared" si="3"/>
         <v>203</v>
       </c>
-    </row>
-    <row r="205" spans="1:1">
+      <c r="B204" t="s">
+        <v>15</v>
+      </c>
+      <c r="L204" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="205" spans="1:12">
       <c r="A205">
         <f t="shared" si="3"/>
         <v>204</v>
       </c>
-    </row>
-    <row r="206" spans="1:1">
+      <c r="B205" t="s">
+        <v>15</v>
+      </c>
+      <c r="L205" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12">
       <c r="A206">
         <f t="shared" si="3"/>
         <v>205</v>
       </c>
-    </row>
-    <row r="207" spans="1:1">
+      <c r="B206" t="s">
+        <v>15</v>
+      </c>
+      <c r="L206" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="207" spans="1:12">
       <c r="A207">
         <f t="shared" si="3"/>
         <v>206</v>
       </c>
-    </row>
-    <row r="208" spans="1:1">
+      <c r="B207" t="s">
+        <v>15</v>
+      </c>
+      <c r="L207" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="208" spans="1:12">
       <c r="A208">
         <f t="shared" si="3"/>
         <v>207</v>
       </c>
-    </row>
-    <row r="209" spans="1:1">
+      <c r="B208" t="s">
+        <v>15</v>
+      </c>
+      <c r="L208" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="209" spans="1:12">
       <c r="A209">
         <f t="shared" si="3"/>
         <v>208</v>
       </c>
-    </row>
-    <row r="210" spans="1:1">
+      <c r="B209" t="s">
+        <v>15</v>
+      </c>
+      <c r="L209" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="210" spans="1:12">
       <c r="A210">
         <f t="shared" si="3"/>
         <v>209</v>
       </c>
-    </row>
-    <row r="211" spans="1:1">
+      <c r="B210" t="s">
+        <v>15</v>
+      </c>
+      <c r="L210" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="211" spans="1:12">
       <c r="A211">
         <f t="shared" si="3"/>
         <v>210</v>
       </c>
-    </row>
-    <row r="212" spans="1:1">
+      <c r="B211" t="s">
+        <v>15</v>
+      </c>
+      <c r="L211" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="212" spans="1:12">
       <c r="A212">
         <f t="shared" si="3"/>
         <v>211</v>
       </c>
-    </row>
-    <row r="213" spans="1:1">
+      <c r="B212" t="s">
+        <v>15</v>
+      </c>
+      <c r="L212" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="213" spans="1:12">
       <c r="A213">
         <f t="shared" si="3"/>
         <v>212</v>
       </c>
-    </row>
-    <row r="214" spans="1:1">
+      <c r="B213" t="s">
+        <v>15</v>
+      </c>
+      <c r="L213" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="214" spans="1:12">
       <c r="A214">
         <f t="shared" si="3"/>
         <v>213</v>
       </c>
-    </row>
-    <row r="215" spans="1:1">
+      <c r="B214" t="s">
+        <v>15</v>
+      </c>
+      <c r="L214" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="215" spans="1:12">
       <c r="A215">
         <f t="shared" si="3"/>
         <v>214</v>
       </c>
-    </row>
-    <row r="216" spans="1:1">
+      <c r="B215" t="s">
+        <v>15</v>
+      </c>
+      <c r="L215" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12">
       <c r="A216">
         <f t="shared" si="3"/>
         <v>215</v>
       </c>
-    </row>
-    <row r="217" spans="1:1">
+      <c r="B216" t="s">
+        <v>15</v>
+      </c>
+      <c r="L216" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="217" spans="1:12">
       <c r="A217">
         <f t="shared" si="3"/>
         <v>216</v>
       </c>
-    </row>
-    <row r="218" spans="1:1">
+      <c r="B217" t="s">
+        <v>15</v>
+      </c>
+      <c r="L217" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12">
       <c r="A218">
         <f t="shared" si="3"/>
         <v>217</v>
       </c>
-    </row>
-    <row r="219" spans="1:1">
+      <c r="B218" t="s">
+        <v>15</v>
+      </c>
+      <c r="L218" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="219" spans="1:12">
       <c r="A219">
         <f t="shared" si="3"/>
         <v>218</v>
       </c>
-    </row>
-    <row r="220" spans="1:1">
+      <c r="B219" t="s">
+        <v>15</v>
+      </c>
+      <c r="L219" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="220" spans="1:12">
       <c r="A220">
         <f t="shared" si="3"/>
         <v>219</v>
       </c>
-    </row>
-    <row r="221" spans="1:1">
+      <c r="B220" t="s">
+        <v>15</v>
+      </c>
+      <c r="L220" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="221" spans="1:12">
       <c r="A221">
         <f t="shared" si="3"/>
         <v>220</v>
       </c>
-    </row>
-    <row r="222" spans="1:1">
+      <c r="B221" t="s">
+        <v>15</v>
+      </c>
+      <c r="L221" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="222" spans="1:12">
       <c r="A222">
         <f t="shared" si="3"/>
         <v>221</v>
       </c>
-    </row>
-    <row r="223" spans="1:1">
+      <c r="B222" t="s">
+        <v>15</v>
+      </c>
+      <c r="L222" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="223" spans="1:12">
       <c r="A223">
         <f t="shared" si="3"/>
         <v>222</v>
       </c>
-    </row>
-    <row r="224" spans="1:1">
+      <c r="B223" t="s">
+        <v>15</v>
+      </c>
+      <c r="L223" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="224" spans="1:12">
       <c r="A224">
         <f t="shared" si="3"/>
         <v>223</v>
       </c>
-    </row>
-    <row r="225" spans="1:1">
+      <c r="B224" t="s">
+        <v>15</v>
+      </c>
+      <c r="L224" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="225" spans="1:12">
       <c r="A225">
         <f t="shared" si="3"/>
         <v>224</v>
       </c>
-    </row>
-    <row r="226" spans="1:1">
+      <c r="B225" t="s">
+        <v>15</v>
+      </c>
+      <c r="L225" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="226" spans="1:12">
       <c r="A226">
         <f t="shared" si="3"/>
         <v>225</v>
       </c>
-    </row>
-    <row r="227" spans="1:1">
+      <c r="B226" t="s">
+        <v>15</v>
+      </c>
+      <c r="L226" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="227" spans="1:12">
       <c r="A227">
         <f t="shared" si="3"/>
         <v>226</v>
       </c>
-    </row>
-    <row r="228" spans="1:1">
+      <c r="B227" t="s">
+        <v>15</v>
+      </c>
+      <c r="L227" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="228" spans="1:12">
       <c r="A228">
         <f t="shared" si="3"/>
         <v>227</v>
       </c>
-    </row>
-    <row r="229" spans="1:1">
+      <c r="B228" t="s">
+        <v>15</v>
+      </c>
+      <c r="L228" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="229" spans="1:12">
       <c r="A229">
         <f t="shared" si="3"/>
         <v>228</v>
       </c>
-    </row>
-    <row r="230" spans="1:1">
+      <c r="B229" t="s">
+        <v>15</v>
+      </c>
+      <c r="L229" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="230" spans="1:12">
       <c r="A230">
         <f t="shared" si="3"/>
         <v>229</v>
       </c>
-    </row>
-    <row r="231" spans="1:1">
+      <c r="B230" t="s">
+        <v>15</v>
+      </c>
+      <c r="L230" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="231" spans="1:12">
       <c r="A231">
         <f t="shared" si="3"/>
         <v>230</v>
       </c>
-    </row>
-    <row r="232" spans="1:1">
+      <c r="B231" t="s">
+        <v>15</v>
+      </c>
+      <c r="L231" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="232" spans="1:12">
       <c r="A232">
         <f t="shared" si="3"/>
         <v>231</v>
       </c>
-    </row>
-    <row r="233" spans="1:1">
+      <c r="B232" t="s">
+        <v>15</v>
+      </c>
+      <c r="L232" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="233" spans="1:12">
       <c r="A233">
         <f t="shared" si="3"/>
         <v>232</v>
       </c>
-    </row>
-    <row r="234" spans="1:1">
+      <c r="B233" t="s">
+        <v>15</v>
+      </c>
+      <c r="L233" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="234" spans="1:12">
       <c r="A234">
         <f t="shared" si="3"/>
         <v>233</v>
       </c>
-    </row>
-    <row r="235" spans="1:1">
+      <c r="B234" t="s">
+        <v>15</v>
+      </c>
+      <c r="L234" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="235" spans="1:12">
       <c r="A235">
         <f t="shared" si="3"/>
         <v>234</v>
       </c>
-    </row>
-    <row r="236" spans="1:1">
+      <c r="B235" t="s">
+        <v>15</v>
+      </c>
+      <c r="L235" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="236" spans="1:12">
       <c r="A236">
         <f t="shared" si="3"/>
         <v>235</v>
       </c>
-    </row>
-    <row r="237" spans="1:1">
+      <c r="B236" t="s">
+        <v>15</v>
+      </c>
+      <c r="L236" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="237" spans="1:12">
       <c r="A237">
         <f t="shared" si="3"/>
         <v>236</v>
       </c>
-    </row>
-    <row r="238" spans="1:1">
+      <c r="B237" t="s">
+        <v>15</v>
+      </c>
+      <c r="L237" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="238" spans="1:12">
       <c r="A238">
         <f t="shared" si="3"/>
         <v>237</v>
       </c>
-    </row>
-    <row r="239" spans="1:1">
+      <c r="B238" t="s">
+        <v>15</v>
+      </c>
+      <c r="L238" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="239" spans="1:12">
       <c r="A239">
         <f t="shared" si="3"/>
         <v>238</v>
       </c>
-    </row>
-    <row r="240" spans="1:1">
+      <c r="B239" t="s">
+        <v>15</v>
+      </c>
+      <c r="L239" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="240" spans="1:12">
       <c r="A240">
         <f t="shared" si="3"/>
         <v>239</v>
       </c>
-    </row>
-    <row r="241" spans="1:1">
+      <c r="B240" t="s">
+        <v>15</v>
+      </c>
+      <c r="L240" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="241" spans="1:12">
       <c r="A241">
         <f t="shared" si="3"/>
         <v>240</v>
       </c>
-    </row>
-    <row r="242" spans="1:1">
+      <c r="B241" t="s">
+        <v>15</v>
+      </c>
+      <c r="L241" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="242" spans="1:12">
       <c r="A242">
         <f t="shared" si="3"/>
         <v>241</v>
       </c>
-    </row>
-    <row r="243" spans="1:1">
+      <c r="B242" t="s">
+        <v>15</v>
+      </c>
+      <c r="L242" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="243" spans="1:12">
       <c r="A243">
         <f t="shared" si="3"/>
         <v>242</v>
       </c>
-    </row>
-    <row r="244" spans="1:1">
+      <c r="B243" t="s">
+        <v>15</v>
+      </c>
+      <c r="L243" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="244" spans="1:12">
       <c r="A244">
         <f t="shared" si="3"/>
         <v>243</v>
       </c>
-    </row>
-    <row r="245" spans="1:1">
+      <c r="B244" t="s">
+        <v>15</v>
+      </c>
+      <c r="L244" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="245" spans="1:12">
       <c r="A245">
         <f t="shared" si="3"/>
         <v>244</v>
       </c>
-    </row>
-    <row r="246" spans="1:1">
+      <c r="B245" t="s">
+        <v>15</v>
+      </c>
+      <c r="L245" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="246" spans="1:12">
       <c r="A246">
         <f t="shared" si="3"/>
         <v>245</v>
       </c>
-    </row>
-    <row r="247" spans="1:1">
+      <c r="B246" t="s">
+        <v>15</v>
+      </c>
+      <c r="L246" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="247" spans="1:12">
       <c r="A247">
         <f t="shared" si="3"/>
         <v>246</v>
       </c>
-    </row>
-    <row r="248" spans="1:1">
+      <c r="B247" t="s">
+        <v>15</v>
+      </c>
+      <c r="L247" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="248" spans="1:12">
       <c r="A248">
         <f t="shared" si="3"/>
         <v>247</v>
       </c>
-    </row>
-    <row r="249" spans="1:1">
+      <c r="B248" t="s">
+        <v>15</v>
+      </c>
+      <c r="L248" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="249" spans="1:12">
       <c r="A249">
         <f t="shared" si="3"/>
         <v>248</v>
       </c>
-    </row>
-    <row r="250" spans="1:1">
+      <c r="B249" t="s">
+        <v>15</v>
+      </c>
+      <c r="L249" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="250" spans="1:12">
       <c r="A250">
         <f t="shared" si="3"/>
         <v>249</v>
       </c>
-    </row>
-    <row r="251" spans="1:1">
+      <c r="B250" t="s">
+        <v>15</v>
+      </c>
+      <c r="L250" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="251" spans="1:12">
       <c r="A251">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-    </row>
-    <row r="252" spans="1:1">
+      <c r="B251" t="s">
+        <v>15</v>
+      </c>
+      <c r="L251" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="252" spans="1:12">
       <c r="A252">
         <f t="shared" si="3"/>
         <v>251</v>
       </c>
-    </row>
-    <row r="253" spans="1:1">
+      <c r="B252" t="s">
+        <v>15</v>
+      </c>
+      <c r="L252" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="253" spans="1:12">
       <c r="A253">
         <f t="shared" si="3"/>
         <v>252</v>
       </c>
-    </row>
-    <row r="254" spans="1:1">
+      <c r="B253" t="s">
+        <v>15</v>
+      </c>
+      <c r="L253" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="254" spans="1:12">
       <c r="A254">
         <f t="shared" si="3"/>
         <v>253</v>
       </c>
-    </row>
-    <row r="255" spans="1:1">
+      <c r="B254" t="s">
+        <v>15</v>
+      </c>
+      <c r="L254" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="255" spans="1:12">
       <c r="A255">
         <f t="shared" si="3"/>
         <v>254</v>
       </c>
-    </row>
-    <row r="256" spans="1:1">
+      <c r="B255" t="s">
+        <v>15</v>
+      </c>
+      <c r="L255" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="256" spans="1:12">
       <c r="A256">
         <f t="shared" si="3"/>
         <v>255</v>
       </c>
-    </row>
-    <row r="257" spans="1:1">
+      <c r="B256" t="s">
+        <v>15</v>
+      </c>
+      <c r="L256" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="257" spans="1:12">
       <c r="A257">
         <f t="shared" si="3"/>
         <v>256</v>
       </c>
-    </row>
-    <row r="258" spans="1:1">
+      <c r="B257" t="s">
+        <v>15</v>
+      </c>
+      <c r="L257" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="258" spans="1:12">
       <c r="A258">
         <f t="shared" si="3"/>
         <v>257</v>
       </c>
-    </row>
-    <row r="259" spans="1:1">
+      <c r="B258" t="s">
+        <v>15</v>
+      </c>
+      <c r="L258" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="259" spans="1:12">
       <c r="A259">
         <f t="shared" si="3"/>
         <v>258</v>
       </c>
-    </row>
-    <row r="260" spans="1:1">
+      <c r="B259" t="s">
+        <v>15</v>
+      </c>
+      <c r="L259" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="260" spans="1:12">
       <c r="A260">
         <f t="shared" ref="A260:A323" si="4">A259+1</f>
         <v>259</v>
       </c>
-    </row>
-    <row r="261" spans="1:1">
+      <c r="B260" t="s">
+        <v>15</v>
+      </c>
+      <c r="L260" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="261" spans="1:12">
       <c r="A261">
         <f t="shared" si="4"/>
         <v>260</v>
       </c>
-    </row>
-    <row r="262" spans="1:1">
+      <c r="B261" t="s">
+        <v>15</v>
+      </c>
+      <c r="L261" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="262" spans="1:12">
       <c r="A262">
         <f t="shared" si="4"/>
         <v>261</v>
       </c>
-    </row>
-    <row r="263" spans="1:1">
+      <c r="B262" t="s">
+        <v>15</v>
+      </c>
+      <c r="L262" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="263" spans="1:12">
       <c r="A263">
         <f t="shared" si="4"/>
         <v>262</v>
       </c>
-    </row>
-    <row r="264" spans="1:1">
+      <c r="B263" t="s">
+        <v>15</v>
+      </c>
+      <c r="L263" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="264" spans="1:12">
       <c r="A264">
         <f t="shared" si="4"/>
         <v>263</v>
       </c>
-    </row>
-    <row r="265" spans="1:1">
+      <c r="B264" t="s">
+        <v>15</v>
+      </c>
+      <c r="L264" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="265" spans="1:12">
       <c r="A265">
         <f t="shared" si="4"/>
         <v>264</v>
       </c>
-    </row>
-    <row r="266" spans="1:1">
+      <c r="B265" t="s">
+        <v>15</v>
+      </c>
+      <c r="L265" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="266" spans="1:12">
       <c r="A266">
         <f t="shared" si="4"/>
         <v>265</v>
       </c>
-    </row>
-    <row r="267" spans="1:1">
+      <c r="B266" t="s">
+        <v>15</v>
+      </c>
+      <c r="L266" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="267" spans="1:12">
       <c r="A267">
         <f t="shared" si="4"/>
         <v>266</v>
       </c>
-    </row>
-    <row r="268" spans="1:1">
+      <c r="B267" t="s">
+        <v>15</v>
+      </c>
+      <c r="L267" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="268" spans="1:12">
       <c r="A268">
         <f t="shared" si="4"/>
         <v>267</v>
       </c>
-    </row>
-    <row r="269" spans="1:1">
+      <c r="B268" t="s">
+        <v>15</v>
+      </c>
+      <c r="L268" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="269" spans="1:12">
       <c r="A269">
         <f t="shared" si="4"/>
         <v>268</v>
       </c>
-    </row>
-    <row r="270" spans="1:1">
+      <c r="B269" t="s">
+        <v>15</v>
+      </c>
+      <c r="L269" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="270" spans="1:12">
       <c r="A270">
         <f t="shared" si="4"/>
         <v>269</v>
       </c>
-    </row>
-    <row r="271" spans="1:1">
+      <c r="B270" t="s">
+        <v>15</v>
+      </c>
+      <c r="L270" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="271" spans="1:12">
       <c r="A271">
         <f t="shared" si="4"/>
         <v>270</v>
       </c>
-    </row>
-    <row r="272" spans="1:1">
+      <c r="B271" t="s">
+        <v>15</v>
+      </c>
+      <c r="L271" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="272" spans="1:12">
       <c r="A272">
         <f t="shared" si="4"/>
         <v>271</v>
       </c>
-    </row>
-    <row r="273" spans="1:1">
+      <c r="B272" t="s">
+        <v>15</v>
+      </c>
+      <c r="L272" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="273" spans="1:12">
       <c r="A273">
         <f t="shared" si="4"/>
         <v>272</v>
       </c>
-    </row>
-    <row r="274" spans="1:1">
+      <c r="B273" t="s">
+        <v>15</v>
+      </c>
+      <c r="L273" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="274" spans="1:12">
       <c r="A274">
         <f t="shared" si="4"/>
         <v>273</v>
       </c>
-    </row>
-    <row r="275" spans="1:1">
+      <c r="B274" t="s">
+        <v>15</v>
+      </c>
+      <c r="L274" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="275" spans="1:12">
       <c r="A275">
         <f t="shared" si="4"/>
         <v>274</v>
       </c>
-    </row>
-    <row r="276" spans="1:1">
+      <c r="B275" t="s">
+        <v>15</v>
+      </c>
+      <c r="L275" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="276" spans="1:12">
       <c r="A276">
         <f t="shared" si="4"/>
         <v>275</v>
       </c>
-    </row>
-    <row r="277" spans="1:1">
+      <c r="B276" t="s">
+        <v>15</v>
+      </c>
+      <c r="L276" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="277" spans="1:12">
       <c r="A277">
         <f t="shared" si="4"/>
         <v>276</v>
       </c>
-    </row>
-    <row r="278" spans="1:1">
+      <c r="B277" t="s">
+        <v>15</v>
+      </c>
+      <c r="L277" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="278" spans="1:12">
       <c r="A278">
         <f t="shared" si="4"/>
         <v>277</v>
       </c>
-    </row>
-    <row r="279" spans="1:1">
+      <c r="B278" t="s">
+        <v>15</v>
+      </c>
+      <c r="L278" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="279" spans="1:12">
       <c r="A279">
         <f t="shared" si="4"/>
         <v>278</v>
       </c>
-    </row>
-    <row r="280" spans="1:1">
+      <c r="B279" t="s">
+        <v>15</v>
+      </c>
+      <c r="L279" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="280" spans="1:12">
       <c r="A280">
         <f t="shared" si="4"/>
         <v>279</v>
       </c>
-    </row>
-    <row r="281" spans="1:1">
+      <c r="B280" t="s">
+        <v>15</v>
+      </c>
+      <c r="L280" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="281" spans="1:12">
       <c r="A281">
         <f t="shared" si="4"/>
         <v>280</v>
       </c>
-    </row>
-    <row r="282" spans="1:1">
+      <c r="B281" t="s">
+        <v>15</v>
+      </c>
+      <c r="L281" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="282" spans="1:12">
       <c r="A282">
         <f t="shared" si="4"/>
         <v>281</v>
       </c>
-    </row>
-    <row r="283" spans="1:1">
+      <c r="B282" t="s">
+        <v>15</v>
+      </c>
+      <c r="L282" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="283" spans="1:12">
       <c r="A283">
         <f t="shared" si="4"/>
         <v>282</v>
       </c>
-    </row>
-    <row r="284" spans="1:1">
+      <c r="B283" t="s">
+        <v>15</v>
+      </c>
+      <c r="L283" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="284" spans="1:12">
       <c r="A284">
         <f t="shared" si="4"/>
         <v>283</v>
       </c>
-    </row>
-    <row r="285" spans="1:1">
+      <c r="B284" t="s">
+        <v>15</v>
+      </c>
+      <c r="L284" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="285" spans="1:12">
       <c r="A285">
         <f t="shared" si="4"/>
         <v>284</v>
       </c>
-    </row>
-    <row r="286" spans="1:1">
+      <c r="B285" t="s">
+        <v>15</v>
+      </c>
+      <c r="L285" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="286" spans="1:12">
       <c r="A286">
         <f t="shared" si="4"/>
         <v>285</v>
       </c>
-    </row>
-    <row r="287" spans="1:1">
+      <c r="B286" t="s">
+        <v>15</v>
+      </c>
+      <c r="L286" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="287" spans="1:12">
       <c r="A287">
         <f t="shared" si="4"/>
         <v>286</v>
       </c>
-    </row>
-    <row r="288" spans="1:1">
+      <c r="B287" t="s">
+        <v>15</v>
+      </c>
+      <c r="L287" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="288" spans="1:12">
       <c r="A288">
         <f t="shared" si="4"/>
         <v>287</v>
       </c>
-    </row>
-    <row r="289" spans="1:1">
+      <c r="B288" t="s">
+        <v>15</v>
+      </c>
+      <c r="L288" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="289" spans="1:12">
       <c r="A289">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
-    </row>
-    <row r="290" spans="1:1">
+      <c r="B289" t="s">
+        <v>15</v>
+      </c>
+      <c r="L289" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="290" spans="1:12">
       <c r="A290">
         <f t="shared" si="4"/>
         <v>289</v>
       </c>
-    </row>
-    <row r="291" spans="1:1">
+      <c r="B290" t="s">
+        <v>15</v>
+      </c>
+      <c r="L290" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="291" spans="1:12">
       <c r="A291">
         <f t="shared" si="4"/>
         <v>290</v>
       </c>
-    </row>
-    <row r="292" spans="1:1">
+      <c r="B291" t="s">
+        <v>15</v>
+      </c>
+      <c r="L291" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="292" spans="1:12">
       <c r="A292">
         <f t="shared" si="4"/>
         <v>291</v>
       </c>
-    </row>
-    <row r="293" spans="1:1">
+      <c r="B292" t="s">
+        <v>15</v>
+      </c>
+      <c r="L292" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="293" spans="1:12">
       <c r="A293">
         <f t="shared" si="4"/>
         <v>292</v>
       </c>
-    </row>
-    <row r="294" spans="1:1">
+      <c r="B293" t="s">
+        <v>15</v>
+      </c>
+      <c r="L293" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="294" spans="1:12">
       <c r="A294">
         <f t="shared" si="4"/>
         <v>293</v>
       </c>
-    </row>
-    <row r="295" spans="1:1">
+      <c r="B294" t="s">
+        <v>15</v>
+      </c>
+      <c r="L294" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="295" spans="1:12">
       <c r="A295">
         <f t="shared" si="4"/>
         <v>294</v>
       </c>
-    </row>
-    <row r="296" spans="1:1">
+      <c r="B295" t="s">
+        <v>15</v>
+      </c>
+      <c r="L295" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="296" spans="1:12">
       <c r="A296">
         <f t="shared" si="4"/>
         <v>295</v>
       </c>
-    </row>
-    <row r="297" spans="1:1">
+      <c r="B296" t="s">
+        <v>15</v>
+      </c>
+      <c r="L296" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="297" spans="1:12">
       <c r="A297">
         <f t="shared" si="4"/>
         <v>296</v>
       </c>
-    </row>
-    <row r="298" spans="1:1">
+      <c r="B297" t="s">
+        <v>15</v>
+      </c>
+      <c r="L297" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="298" spans="1:12">
       <c r="A298">
         <f t="shared" si="4"/>
         <v>297</v>
       </c>
-    </row>
-    <row r="299" spans="1:1">
+      <c r="B298" t="s">
+        <v>15</v>
+      </c>
+      <c r="L298" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="299" spans="1:12">
       <c r="A299">
         <f t="shared" si="4"/>
         <v>298</v>
       </c>
-    </row>
-    <row r="300" spans="1:1">
+      <c r="B299" t="s">
+        <v>15</v>
+      </c>
+      <c r="L299" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="300" spans="1:12">
       <c r="A300">
         <f t="shared" si="4"/>
         <v>299</v>
       </c>
-    </row>
-    <row r="301" spans="1:1">
+      <c r="B300" t="s">
+        <v>15</v>
+      </c>
+      <c r="L300" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="301" spans="1:12">
       <c r="A301">
         <f t="shared" si="4"/>
         <v>300</v>
       </c>
-    </row>
-    <row r="302" spans="1:1">
+      <c r="B301" t="s">
+        <v>15</v>
+      </c>
+      <c r="L301" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="302" spans="1:12">
       <c r="A302">
         <f t="shared" si="4"/>
         <v>301</v>
       </c>
-    </row>
-    <row r="303" spans="1:1">
+      <c r="B302" t="s">
+        <v>15</v>
+      </c>
+      <c r="L302" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="303" spans="1:12">
       <c r="A303">
         <f t="shared" si="4"/>
         <v>302</v>
       </c>
-    </row>
-    <row r="304" spans="1:1">
+      <c r="B303" t="s">
+        <v>15</v>
+      </c>
+      <c r="L303" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="304" spans="1:12">
       <c r="A304">
         <f t="shared" si="4"/>
         <v>303</v>
       </c>
-    </row>
-    <row r="305" spans="1:1">
+      <c r="B304" t="s">
+        <v>15</v>
+      </c>
+      <c r="L304" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="305" spans="1:12">
       <c r="A305">
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-    </row>
-    <row r="306" spans="1:1">
+      <c r="B305" t="s">
+        <v>15</v>
+      </c>
+      <c r="L305" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="306" spans="1:12">
       <c r="A306">
         <f t="shared" si="4"/>
         <v>305</v>
       </c>
-    </row>
-    <row r="307" spans="1:1">
+      <c r="B306" t="s">
+        <v>15</v>
+      </c>
+      <c r="L306" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="307" spans="1:12">
       <c r="A307">
         <f t="shared" si="4"/>
         <v>306</v>
       </c>
-    </row>
-    <row r="308" spans="1:1">
+      <c r="B307" t="s">
+        <v>15</v>
+      </c>
+      <c r="L307" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="308" spans="1:12">
       <c r="A308">
         <f t="shared" si="4"/>
         <v>307</v>
       </c>
-    </row>
-    <row r="309" spans="1:1">
+      <c r="B308" t="s">
+        <v>15</v>
+      </c>
+      <c r="L308" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="309" spans="1:12">
       <c r="A309">
         <f t="shared" si="4"/>
         <v>308</v>
       </c>
-    </row>
-    <row r="310" spans="1:1">
+      <c r="B309" t="s">
+        <v>15</v>
+      </c>
+      <c r="L309" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="310" spans="1:12">
       <c r="A310">
         <f t="shared" si="4"/>
         <v>309</v>
       </c>
-    </row>
-    <row r="311" spans="1:1">
+      <c r="B310" t="s">
+        <v>15</v>
+      </c>
+      <c r="L310" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="311" spans="1:12">
       <c r="A311">
         <f t="shared" si="4"/>
         <v>310</v>
       </c>
-    </row>
-    <row r="312" spans="1:1">
+      <c r="B311" t="s">
+        <v>15</v>
+      </c>
+      <c r="L311" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="312" spans="1:12">
       <c r="A312">
         <f t="shared" si="4"/>
         <v>311</v>
       </c>
-    </row>
-    <row r="313" spans="1:1">
+      <c r="B312" t="s">
+        <v>15</v>
+      </c>
+      <c r="L312" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="313" spans="1:12">
       <c r="A313">
         <f t="shared" si="4"/>
         <v>312</v>
       </c>
-    </row>
-    <row r="314" spans="1:1">
+      <c r="B313" t="s">
+        <v>15</v>
+      </c>
+      <c r="L313" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="314" spans="1:12">
       <c r="A314">
         <f t="shared" si="4"/>
         <v>313</v>
       </c>
-    </row>
-    <row r="315" spans="1:1">
+      <c r="B314" t="s">
+        <v>15</v>
+      </c>
+      <c r="L314" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="315" spans="1:12">
       <c r="A315">
         <f t="shared" si="4"/>
         <v>314</v>
       </c>
-    </row>
-    <row r="316" spans="1:1">
+      <c r="B315" t="s">
+        <v>15</v>
+      </c>
+      <c r="L315" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="316" spans="1:12">
       <c r="A316">
         <f t="shared" si="4"/>
         <v>315</v>
       </c>
-    </row>
-    <row r="317" spans="1:1">
+      <c r="B316" t="s">
+        <v>15</v>
+      </c>
+      <c r="L316" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="317" spans="1:12">
       <c r="A317">
         <f t="shared" si="4"/>
         <v>316</v>
       </c>
-    </row>
-    <row r="318" spans="1:1">
+      <c r="B317" t="s">
+        <v>15</v>
+      </c>
+      <c r="L317" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="318" spans="1:12">
       <c r="A318">
         <f t="shared" si="4"/>
         <v>317</v>
       </c>
-    </row>
-    <row r="319" spans="1:1">
+      <c r="B318" t="s">
+        <v>15</v>
+      </c>
+      <c r="L318" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="319" spans="1:12">
       <c r="A319">
         <f t="shared" si="4"/>
         <v>318</v>
       </c>
-    </row>
-    <row r="320" spans="1:1">
+      <c r="B319" t="s">
+        <v>15</v>
+      </c>
+      <c r="L319" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="320" spans="1:12">
       <c r="A320">
         <f t="shared" si="4"/>
         <v>319</v>
       </c>
-    </row>
-    <row r="321" spans="1:1">
+      <c r="B320" t="s">
+        <v>15</v>
+      </c>
+      <c r="L320" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="321" spans="1:12">
       <c r="A321">
         <f t="shared" si="4"/>
         <v>320</v>
       </c>
-    </row>
-    <row r="322" spans="1:1">
+      <c r="B321" t="s">
+        <v>15</v>
+      </c>
+      <c r="L321" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="322" spans="1:12">
       <c r="A322">
         <f t="shared" si="4"/>
         <v>321</v>
       </c>
-    </row>
-    <row r="323" spans="1:1">
+      <c r="B322" t="s">
+        <v>15</v>
+      </c>
+      <c r="L322" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="323" spans="1:12">
       <c r="A323">
         <f t="shared" si="4"/>
         <v>322</v>
       </c>
-    </row>
-    <row r="324" spans="1:1">
+      <c r="B323" t="s">
+        <v>15</v>
+      </c>
+      <c r="L323" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="324" spans="1:12">
       <c r="A324">
         <f t="shared" ref="A324:A330" si="5">A323+1</f>
         <v>323</v>
       </c>
-    </row>
-    <row r="325" spans="1:1">
+      <c r="B324" t="s">
+        <v>15</v>
+      </c>
+      <c r="L324" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="325" spans="1:12">
       <c r="A325">
         <f t="shared" si="5"/>
         <v>324</v>
       </c>
-    </row>
-    <row r="326" spans="1:1">
+      <c r="B325" t="s">
+        <v>15</v>
+      </c>
+      <c r="L325" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="326" spans="1:12">
       <c r="A326">
         <f t="shared" si="5"/>
         <v>325</v>
       </c>
-    </row>
-    <row r="327" spans="1:1">
+      <c r="B326" t="s">
+        <v>15</v>
+      </c>
+      <c r="L326" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="327" spans="1:12">
       <c r="A327">
         <f t="shared" si="5"/>
         <v>326</v>
       </c>
-    </row>
-    <row r="328" spans="1:1">
+      <c r="B327" t="s">
+        <v>15</v>
+      </c>
+      <c r="L327" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="328" spans="1:12">
       <c r="A328">
         <f t="shared" si="5"/>
         <v>327</v>
       </c>
-    </row>
-    <row r="329" spans="1:1">
+      <c r="B328" t="s">
+        <v>15</v>
+      </c>
+      <c r="L328" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="329" spans="1:12">
       <c r="A329">
         <f t="shared" si="5"/>
         <v>328</v>
       </c>
-    </row>
-    <row r="330" spans="1:1">
+      <c r="B329" t="s">
+        <v>15</v>
+      </c>
+      <c r="L329" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="330" spans="1:12">
       <c r="A330">
         <f t="shared" si="5"/>
         <v>329</v>
+      </c>
+      <c r="B330" t="s">
+        <v>15</v>
+      </c>
+      <c r="L330" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished the templates for seminoles
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Creek/Creek Freedman Minor.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Creek/Creek Freedman Minor.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="24">
   <si>
     <t>ID</t>
   </si>
@@ -80,6 +80,12 @@
   </si>
   <si>
     <t>Image Binary</t>
+  </si>
+  <si>
+    <t>Stricken from roll</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -5638,8 +5644,35 @@
         <f t="shared" si="12"/>
         <v>615</v>
       </c>
+      <c r="D260" t="s">
+        <v>22</v>
+      </c>
+      <c r="E260" t="s">
+        <v>23</v>
+      </c>
+      <c r="F260" t="s">
+        <v>23</v>
+      </c>
+      <c r="G260" t="s">
+        <v>23</v>
+      </c>
+      <c r="H260">
+        <v>-1</v>
+      </c>
+      <c r="I260" t="s">
+        <v>23</v>
+      </c>
+      <c r="J260" t="s">
+        <v>23</v>
+      </c>
+      <c r="K260" t="s">
+        <v>23</v>
+      </c>
       <c r="L260" t="s">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="M260" t="s">
+        <v>23</v>
       </c>
       <c r="N260" t="str">
         <f t="shared" si="13"/>
@@ -5658,8 +5691,35 @@
         <f t="shared" si="12"/>
         <v>615</v>
       </c>
+      <c r="D261" t="s">
+        <v>22</v>
+      </c>
+      <c r="E261" t="s">
+        <v>23</v>
+      </c>
+      <c r="F261" t="s">
+        <v>23</v>
+      </c>
+      <c r="G261" t="s">
+        <v>23</v>
+      </c>
+      <c r="H261">
+        <v>0</v>
+      </c>
+      <c r="I261" t="s">
+        <v>23</v>
+      </c>
+      <c r="J261" t="s">
+        <v>23</v>
+      </c>
+      <c r="K261" t="s">
+        <v>23</v>
+      </c>
       <c r="L261" t="s">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="M261" t="s">
+        <v>23</v>
       </c>
       <c r="N261" t="str">
         <f t="shared" si="13"/>
@@ -5678,8 +5738,35 @@
         <f t="shared" si="12"/>
         <v>615</v>
       </c>
+      <c r="D262" t="s">
+        <v>22</v>
+      </c>
+      <c r="E262" t="s">
+        <v>23</v>
+      </c>
+      <c r="F262" t="s">
+        <v>23</v>
+      </c>
+      <c r="G262" t="s">
+        <v>23</v>
+      </c>
+      <c r="H262">
+        <v>1</v>
+      </c>
+      <c r="I262" t="s">
+        <v>23</v>
+      </c>
+      <c r="J262" t="s">
+        <v>23</v>
+      </c>
+      <c r="K262" t="s">
+        <v>23</v>
+      </c>
       <c r="L262" t="s">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="M262" t="s">
+        <v>23</v>
       </c>
       <c r="N262" t="str">
         <f t="shared" si="13"/>

</xml_diff>